<commit_message>
7 step of analyses and table to show output
</commit_message>
<xml_diff>
--- a/Parameters and variables.xlsx
+++ b/Parameters and variables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Safi\Documents\GitHub\THEE-Fragmentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7A4310-8FAD-493F-8F9F-9CB648FB6BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C107D2F7-DB14-402E-9E0B-F39869169622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4890" yWindow="0" windowWidth="14400" windowHeight="10170" xr2:uid="{DE916E10-2DE2-462D-8716-E75A7ABC8A34}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DE916E10-2DE2-462D-8716-E75A7ABC8A34}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="47">
   <si>
     <t>THEE Model</t>
   </si>
@@ -156,6 +156,30 @@
   </si>
   <si>
     <t>limiting growth of the populations, same proportion as habitat</t>
+  </si>
+  <si>
+    <t>Model outcomes</t>
+  </si>
+  <si>
+    <t>Evolutionary rescue</t>
+  </si>
+  <si>
+    <t>Habitat A</t>
+  </si>
+  <si>
+    <t>Habitat B</t>
+  </si>
+  <si>
+    <t>Habitat C</t>
+  </si>
+  <si>
+    <t>Habitat B&amp;C</t>
+  </si>
+  <si>
+    <t>Before split_time</t>
+  </si>
+  <si>
+    <t>After split_time</t>
   </si>
 </sst>
 </file>
@@ -171,15 +195,45 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -187,12 +241,147 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -527,25 +716,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5DC6963-9A1E-4816-942E-6A33061D1B7A}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.81640625" customWidth="1"/>
     <col min="3" max="3" width="51.453125" customWidth="1"/>
     <col min="4" max="4" width="13.7265625" customWidth="1"/>
+    <col min="6" max="6" width="17.26953125" customWidth="1"/>
+    <col min="12" max="12" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F1" s="6"/>
+      <c r="G1" s="9"/>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2" s="6"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -558,8 +758,19 @@
       <c r="D3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3" s="6"/>
+      <c r="F3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="11"/>
+      <c r="L3" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -572,8 +783,24 @@
       <c r="D4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -586,8 +813,15 @@
       <c r="D5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="14"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -600,8 +834,16 @@
       <c r="D6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6" s="13"/>
+      <c r="F6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -614,8 +856,14 @@
       <c r="D7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7" s="13"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -628,8 +876,14 @@
       <c r="D8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8" s="13"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -643,7 +897,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -657,7 +911,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -671,7 +925,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -685,7 +939,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -699,7 +953,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>30</v>
       </c>

</xml_diff>